<commit_message>
docs(X-11): check „API unit tests" dopisany do rulesetu
Rozdzielenie jobów bez tego kroku OTWIERAŁO dziurę: testy byłyby widoczne, ale
niewymagane do scalenia, więc PR z czerwonymi testami przeszedłby, gdyby
pozostałe trzy checki były zielone. Zmiana poprawiająca widoczność kosztem
egzekwowania jest gorsza niż stan wyjściowy — dlatego oba kroki należą do
jednego zadania.

Ruleset 21161479 wymaga teraz czterech checków:
  Static checks (lint + typecheck)
  Build (api + panels)
  Prisma migrate deploy (smoke)
  API unit tests

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GiC39BUJm2q9fBrGMwDUiv
</commit_message>
<xml_diff>
--- a/audyt-parytetu-2026-08/VERRIS_PARYTET_FUNKCJI_2026-08.xlsx
+++ b/audyt-parytetu-2026-08/VERRIS_PARYTET_FUNKCJI_2026-08.xlsx
@@ -26035,7 +26035,7 @@
       </c>
       <c r="J349" s="12" t="inlineStr">
         <is>
-          <t>ruleset „gałęzie wdrożeniowe — wymagaj zielonego CI" (id 21161479), Active, zakres: gałąź domyślna + live-release-readiness; wymagane 3 checki z ci.yml</t>
+          <t>ruleset „gałęzie wdrożeniowe — wymagaj zielonego CI" (id 21161479), Active, zakres: gałąź domyślna + live-release-readiness; wymagane 4 checki z ci.yml</t>
         </is>
       </c>
       <c r="K349" s="11" t="inlineStr">
@@ -26695,7 +26695,7 @@
       </c>
       <c r="N358" s="12" t="inlineStr">
         <is>
-          <t>Zamknięte 2026-08-21. Zasada: krok, który DOWODZI, nie może stać za krokiem, który tylko sprawdza higienę. Przy przebiegu #17 typecheck wywalił się na apps/www — panelu niezwiązanym z tamtą pracą — i 194 testy nie uruchomiły się ani razu. Koszt rozdzielenia: jeden dodatkowy pnpm install, joby i tak biegną równolegle. deploy.yml celowo zostaje z testami w jednym jobie z typecheckiem, bo zadaniem bramki jest zablokować wdrożenie, a nie dostarczyć dowód. UWAGA: nowy check trzeba dopisać do rulesetu z X-02, inaczej nie jest wymagany do scalenia. Dokumentacja: docs/zadania/X-11-testy-api-w-osobnym-jobie.md</t>
+          <t>Zamknięte 2026-08-21. Zasada: krok, który DOWODZI, nie może stać za krokiem, który tylko sprawdza higienę. Przy przebiegu #17 typecheck wywalił się na apps/www — panelu niezwiązanym z tamtą pracą — i 194 testy nie uruchomiły się ani razu. Koszt rozdzielenia: jeden dodatkowy pnpm install, joby i tak biegną równolegle. deploy.yml celowo zostaje z testami w jednym jobie z typecheckiem, bo zadaniem bramki jest zablokować wdrożenie, a nie dostarczyć dowód. Check „API unit tests" dopisany do rulesetu z X-02 tego samego dnia — bez tego rozdzielenie jobów otwierałoby dziurę: testy widoczne, ale niewymagane do scalenia. Dokumentacja: docs/zadania/X-11-testy-api-w-osobnym-jobie.md</t>
         </is>
       </c>
     </row>

</xml_diff>